<commit_message>
feat: update anomaly banner and add daily 6 PM auto update scheduler
</commit_message>
<xml_diff>
--- a/spread.xlsx
+++ b/spread.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1229"/>
+  <dimension ref="A1:J1230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -42271,6 +42271,40 @@
         <v>0.396</v>
       </c>
     </row>
+    <row r="1230">
+      <c r="A1230" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B1230" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C1230" s="3" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="D1230" s="3" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="E1230" s="3" t="n">
+        <v>4.386</v>
+      </c>
+      <c r="F1230" s="3" t="n">
+        <v>1.886</v>
+      </c>
+      <c r="G1230" s="3" t="n">
+        <v>3.239</v>
+      </c>
+      <c r="H1230" s="3" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="I1230" s="3" t="n">
+        <v>2.893</v>
+      </c>
+      <c r="J1230" s="3" t="n">
+        <v>0.393</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>